<commit_message>
Costs in the viewers (cost fact from docs/costs/costs.json) and an itemized cost section for the setup page; rover sliced PETG and hours in the cost model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EEyVHbLyBsmH2svqtVnwY7
</commit_message>
<xml_diff>
--- a/docs/costs/robot_build_costs.xlsx
+++ b/docs/costs/robot_build_costs.xlsx
@@ -9097,7 +9097,7 @@
         </is>
       </c>
       <c r="D42" s="29" t="n">
-        <v>0.303</v>
+        <v>0.335</v>
       </c>
       <c r="E42" s="8">
         <f>Summary!$C$9</f>
@@ -9117,7 +9117,7 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Round-2 slices; round 3 not sliced yet. 'Cost to buy' counts whole 1 kg spools.</t>
+          <t>Slices of 26 Oct 2026: 8 plates (chassis round 6, lid, sprockets, idlers, wheels 2 x 2, links 35 x 2). 'Cost to buy' counts whole 1 kg spools.</t>
         </is>
       </c>
     </row>
@@ -9133,7 +9133,7 @@
         </is>
       </c>
       <c r="D43" s="29" t="n">
-        <v>30.4</v>
+        <v>33</v>
       </c>
       <c r="E43" s="31">
         <f>Summary!$C$11*Summary!$C$10</f>

</xml_diff>